<commit_message>
feat(F-NAR-019): ATOM-DIF.BES.001-04 Les cubes de Nino
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.BES.001-04.xlsx
+++ b/stories/arbres/ATOM-DIF.BES.001-04.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>La tour de Nino</t>
+          <t>Les cubes de Nino</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>salon, tapis, canapé</t>
+          <t>salon. Rayon jaune sur tapis, cube sous canapé, horloge, pain du goûter</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Nino, Victorina, papa, maman</t>
+          <t>Nino, papa, maman</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Nino veut une tour qui touche le rayon. Victorina reste près du canapé. Il répète. Elle observe d'abord. Un cube, puis la tour.</t>
+          <t>Un rayon jaune pose un carré sur le tapis. Sur l'arête, un éclat de cube luit. Nino veut une tour, maintenant, aussi haute que le canapé. Il prend trop de cubes : clac, la tour tombe. Le cube jaune roule sous le canapé. Sourire parti. Papa se baisse. Nino pose un cube, puis un autre. Merci vécu. Sous le canapé, la main trop vite : le cube glisse. Il refuse de foncer. Sur l'arête, l'éclat de cube tient.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Le doudou a glissé entre deux coussins. Une oreille dépasse, toute molle. Ça sent le cacao du goûter, encore. L'horloge pose un tic, puis un tac. Un cube rouge brille près du canapé. Tu as vu l'oreille, Nino ? Le doudou attend. Oui. Entre les coussins. Je veux une tour. Qui touche la lumière. Une tour de cubes, alors. Un rayon passe sur le tapis. Il est pâle, un peu long. Le rideau bouge un peu. Tu as vu le rideau ? Il fait du vent. Un tout petit vent. En ce moment, Nino est au salon. D'autres cubes sont là. Bleus. Verts. Ils sont lisses, un peu froids. Victorina reste près du canapé. Elle tient le bord du tissu. Victorina. Tu viens ? Victorina ne vient pas encore. Elle a besoin de calme. Tu peux dire comment on pose. Le cube jaune se cache sous le canapé. Le rayon attend sur le tapis.</t>
+          <t>Un rayon jaune pose un carré sur le tapis. Le pied du canapé le coupe. Un cube jaune y reste coincé. Sur l'arête, un éclat de cube luit. Il brille, papa. Tu le vois, sur le cube ? Ça sent le pain du goûter. Papa coupe le pain, près de la table. L'horloge fait tic-tac. Le rideau bouge un peu. Un doudou attend sur le canapé. Tu as vu le cube, Nino ? Il est sous le canapé. On le laisse un moment. D'autres cubes sont sur le tapis. Ils sont lisses, un peu froids. Un bleu attend près du pied. Je veux une tour, maintenant ! Aussi haute que le canapé ! Tu la veux vite ? Oui, tout de suite ! En ce moment, Nino prend trop de cubes. Les cubes glissent entre ses doigts. Ça fait clac, sur le tapis. La tour tombe, trop vite. Le cube jaune roule sous le canapé. Oh. L'éclat de cube tremble, puis tient. Le sourire de Nino disparaît. Dans sa poitrine, ça se bouscule. L'envie et l'inquiétude se heurtent. Ça ne veut pas, papa. Ses épaules tombent un peu. Papa se baisse à sa hauteur. Tu regardes les cubes ? Je les veux tous. Tu les prends trop vite, Nino ? Oui, maman. Nino serre les mains, trop fort. Ses doigts restent fermés. Son souffle est court. On regarde un cube ? Un seul ?</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Le doudou a glissé entre deux coussins. Une oreille dépasse, toute molle. Ça sent le cacao du goûter, encore. L'horloge pose un tic, puis un tac. Un cube rouge brille près du canapé. Tu as vu l'oreille, Nino ? Le doudou attend. Oui. Entre les coussins. Je veux une tour. Qui touche la lumière. Une tour de cubes, alors. Un rayon passe sur le tapis. Il est pâle, un peu long. Le rideau bouge un peu. Tu as vu le rideau ? Il fait du vent. Un tout petit vent. En ce moment, Nino est au salon. D'autres cubes sont là. Bleus. Verts. Ils sont lisses, un peu froids. Victorina reste près du canapé. Elle tient le bord du tissu. Victorina. Tu viens ? Victorina ne vient pas encore. Elle a besoin de calme. Tu peux dire comment on pose. Le cube jaune se cache sous le canapé. Le rayon attend sur le tapis.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Un rayon jaune pose un carré sur le tapis. Le pied du canapé le coupe. Un cube jaune y reste coincé. Sur l'arête, un &lt;emphasis level="moderate"&gt;éclat de cube&lt;/emphasis&gt; luit. Il brille, papa. Tu le vois, sur le cube ? Ça sent le pain du goûter. Papa coupe le pain, près de la table. L'horloge fait tic-tac. Le rideau bouge un peu. Un doudou attend sur le canapé. Tu as vu le cube, Nino ? Il est sous le canapé. On le laisse un moment. D'autres cubes sont sur le tapis. Ils sont lisses, un peu froids. Un bleu attend près du pied. Je veux une tour, maintenant ! Aussi haute que le canapé ! Tu la veux vite ? Oui, tout de suite ! En ce moment, Nino prend trop de cubes. Les cubes glissent entre ses doigts. Ça fait clac, sur le tapis. La tour tombe, trop vite. Le cube jaune roule sous le canapé. Oh. L'éclat de cube tremble, puis tient. Le sourire de Nino disparaît. Dans sa poitrine, ça se bouscule. L'envie et l'inquiétude se heurtent. Ça ne veut pas, papa. Ses épaules tombent un peu. Papa se baisse à sa hauteur. Tu regardes les cubes ? Je les veux tous. Tu les prends trop vite, Nino ? Oui, maman. Nino serre les mains, trop fort. Ses doigts restent fermés. Son souffle est court. On regarde un cube ? Un seul ?&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Bérénice est au salon. Maman est là. Clément est là aussi. Il y a des cubes. Maman dit la règle. On pose un cube. Puis un autre cube. Tout doux. Clément reste près du canapé. Il a besoin de calme. Bérénice l'appelle. Clément ne vient pas. Maman dit : on peut &lt;emphasis&gt;répéter&lt;/emphasis&gt;. On peut observer d'abord. Bérénice va près de Clément. Elle parle doucement. Bérénice dit : un cube. Puis un autre. C'est répéter. Clément écoute. Il va observer d'abord. Bérénice pose un cube. Clément regarde. Il ne joue pas encore. C'est possible. Maman dit : Clément peut observer d'abord. Bérénice continue. Elle pose un cube bleu. Clément sourit un peu. Plus tard, Clément tend la main. Il pose un cube. Bérénice laisse l'espace. Maman dit : tu as su répéter. Clément a pu observer d'abord.&lt;/slow&gt; [pause]</t>
+          <t>Un rayon jaune pose un carré sur le tapis. Le pied du canapé le coupe. Un cube jaune y reste coincé. Sur l'arête, un &lt;emphasis&gt;éclat de cube&lt;/emphasis&gt; luit. Il brille, papa. Tu le vois, sur le cube ? Ça sent le pain du goûter. Papa coupe le pain, près de la table. L'horloge fait tic-tac. Le rideau bouge un peu. Un doudou attend sur le canapé. Tu as vu le cube, Nino ? Il est sous le canapé. On le laisse un moment. D'autres cubes sont sur le tapis. Ils sont lisses, un peu froids. Un bleu attend près du pied. Je veux une tour, maintenant ! Aussi haute que le canapé ! Tu la veux vite ? Oui, tout de suite ! En ce moment, Nino prend trop de cubes. Les cubes glissent entre ses doigts. Ça fait clac, sur le tapis. La tour tombe, trop vite. Le cube jaune roule sous le canapé. Oh. L'éclat de cube tremble, puis tient. Le sourire de Nino disparaît. Dans sa poitrine, ça se bouscule. L'envie et l'inquiétude se heurtent. Ça ne veut pas, papa. Ses épaules tombent un peu. Papa se baisse à sa hauteur. Tu regardes les cubes ? Je les veux tous. Tu les prends trop vite, Nino ? Oui, maman. Nino serre les mains, trop fort. Ses doigts restent fermés. Son souffle est court. On regarde un cube ? Un seul ? [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,18 +1246,18 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>118</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.28</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>répéter</t>
+          <t>éclat de cube</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>380</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1324,43 +1324,58 @@
         <v>50</v>
       </c>
       <c r="AU2" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=il_veut_la_tour_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Le doudou a glissé entre deux coussins.
-narrateur|Une oreille dépasse, toute molle.
-narrateur|Ça sent le cacao du goûter, encore.
-narrateur|L'horloge pose un tic, puis un tac.
-narrateur|Un cube rouge brille près du canapé.
-maman|Tu as vu l'oreille, Nino ?
-enfant-m|Le doudou attend.
-maman|Oui.
-maman|Entre les coussins.
-enfant-m|Je veux une tour.
-enfant-m|Qui touche la lumière.
-maman|Une tour de cubes, alors.
-narrateur|Un rayon passe sur le tapis.
-narrateur|Il est pâle, un peu long.
+          <t>narrateur|Un rayon jaune pose un carré sur le tapis.
+narrateur|Le pied du canapé le coupe.
+narrateur|Un cube jaune y reste coincé.
+narrateur|Sur l'arête, un éclat de cube luit.
+enfant-m|Il brille, papa.
+papa|Tu le vois, sur le cube ?
+narrateur|Ça sent le pain du goûter.
+narrateur|Papa coupe le pain, près de la table.
+narrateur|L'horloge fait tic-tac.
 narrateur|Le rideau bouge un peu.
-maman|Tu as vu le rideau ?
-enfant-m|Il fait du vent.
-maman|Un tout petit vent.
-narrateur|En ce moment, Nino est au salon.
-narrateur|D'autres cubes sont là.
-narrateur|Bleus.
-narrateur|Verts.
+narrateur|Un doudou attend sur le canapé.
+maman|Tu as vu le cube, Nino ?
+enfant-m|Il est sous le canapé.
+maman|On le laisse un moment.
+narrateur|D'autres cubes sont sur le tapis.
 narrateur|Ils sont lisses, un peu froids.
-narrateur|Victorina reste près du canapé.
-narrateur|Elle tient le bord du tissu.
-enfant-m|Victorina.
-enfant-m|Tu viens ?
-narrateur|Victorina ne vient pas encore.
-maman|Elle a besoin de calme.
-maman|Tu peux dire comment on pose.
-narrateur|Le cube jaune se cache sous le canapé.
-narrateur|Le rayon attend sur le tapis.</t>
+narrateur|Un bleu attend près du pied.
+enfant-m|Je veux une tour, maintenant !
+enfant-m|Aussi haute que le canapé !
+papa|Tu la veux vite ?
+enfant-m|Oui, tout de suite !
+narrateur|En ce moment, Nino prend trop de cubes.
+narrateur|Les cubes glissent entre ses doigts.
+narrateur|Ça fait clac, sur le tapis.
+narrateur|La tour tombe, trop vite.
+narrateur|Le cube jaune roule sous le canapé.
+enfant-m|Oh.
+narrateur|L'éclat de cube tremble, puis tient.
+narrateur|Le sourire de Nino disparaît.
+narrateur|Dans sa poitrine, ça se bouscule.
+narrateur|L'envie et l'inquiétude se heurtent.
+enfant-m|Ça ne veut pas, papa.
+narrateur|Ses épaules tombent un peu.
+narrateur|Papa se baisse à sa hauteur.
+papa|Tu regardes les cubes ?
+enfant-m|Je les veux tous.
+maman|Tu les prends trop vite, Nino ?
+enfant-m|Oui, maman.
+narrateur|Nino serre les mains, trop fort.
+narrateur|Ses doigts restent fermés.
+narrateur|Son souffle est court.
+papa|On regarde un cube ?
+enfant-m|Un seul ?</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1392,17 +1407,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Victorina a besoin de calme. Que peut-on faire ?</t>
+          <t>Nino a besoin de calme. Que peut-on faire ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Victorina a besoin de calme. Que peut-on faire ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Nino a besoin de &lt;emphasis level="moderate"&gt;calme&lt;/emphasis&gt;. Que peut-on faire ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Clément a besoin de calme. Que peut-on faire ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Nino a besoin de &lt;emphasis&gt;calme&lt;/emphasis&gt;. Que peut-on faire ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1465,7 +1480,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1473,10 +1488,10 @@
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.4</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1491,34 +1506,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>380</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1527,13 +1546,13 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
@@ -1543,12 +1562,12 @@
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=nino_a_besoin_de_calme_on_peut_repeter; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Victorina a besoin de calme.
+          <t>narrateur|Nino a besoin de calme.
 narrateur|Que peut-on faire ?</t>
         </is>
       </c>
@@ -1576,17 +1595,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Nino va près du canapé. Il parle tout doux. Un cube. Puis un autre. Tout doux. Tu as su répéter. Victorina écoute. Elle va observer d'abord. Nino pose un cube bleu. Le cube fait un petit bruit. Victorina regarde. Observer d'abord, c'est possible. Nino pose un cube vert. La tour monte un peu. Plus tard, Victorina tend la main. Elle pose le cube rouge. Encore un. Nino glisse le cube jaune. Celui du canapé. Il le pose tout en haut. La tour touche le rayon. Bravo, Nino. Tu as laissé le temps. Elle touche la lumière. Oui. Le cube jaune brille un peu. Victorina pose une main à plat. On n'avance plus. On regarde, maintenant.</t>
+          <t>Nino referme la bouche. Il refuse de tout prendre. Personne ne parle. Il observe un cube bleu. Il écoute le salon, un instant. Un cube. Nino pose le cube bleu. Le tapis le tient. Puis un autre. Il pose un cube rouge. Le même geste, deux fois. Tu poses un, puis un ? Oui, papa. La petite tour tient. Merci, Nino. Papa a vu le geste entier. Le ventre de Nino se desserre. Les épaules se relèvent un peu. Elle tient, maman. Tu la vois, ta tour ? Oui, maman. Le cube jaune reste sous le canapé. Je le vois, là. Il attend, sous le bois ? Oui. Nino ne tend pas la main. Il reste près de sa tour.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Nino va près du canapé. Il parle tout doux. Un cube. Puis un autre. Tout doux. Tu as su répéter. Victorina écoute. Elle va observer d'abord. Nino pose un cube bleu. Le cube fait un petit bruit. Victorina regarde. Observer d'abord, c'est possible. Nino pose un cube vert. La tour monte un peu. Plus tard, Victorina tend la main. Elle pose le cube rouge. Encore un. Nino glisse le cube jaune. Celui du canapé. Il le pose tout en haut. La tour touche le rayon. Bravo, Nino. Tu as laissé le temps. Elle touche la lumière. Oui. Le cube jaune brille un peu. Victorina pose une main à plat. On n'avance plus. On regarde, maintenant.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino referme la bouche. Il refuse de tout prendre. Personne ne parle. Il observe un &lt;emphasis level="moderate"&gt;cube&lt;/emphasis&gt; bleu. Il écoute le salon, un instant. Un cube. Nino pose le cube bleu. Le tapis le tient. Puis un autre. Il pose un cube rouge. Le même geste, deux fois. Tu poses un, puis un ? Oui, papa. La petite tour tient. Merci, Nino. Papa a vu le geste entier. Le ventre de Nino se desserre. Les épaules se relèvent un peu. Elle tient, maman. Tu la vois, ta tour ? Oui, maman. Le cube jaune reste sous le canapé. Je le vois, là. Il attend, sous le bois ? Oui. Nino ne tend pas la main. Il reste près de sa tour.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Bérénice a su &lt;emphasis&gt;répéter&lt;/emphasis&gt;. Clément a pu observer d'abord. Le jeu a continué.&lt;/slow&gt; [pause]</t>
+          <t>Nino referme la bouche. Il refuse de tout prendre. Personne ne parle. Il observe un &lt;emphasis&gt;cube&lt;/emphasis&gt; bleu. Il écoute le salon, un instant. Un cube. Nino pose le cube bleu. Le tapis le tient. Puis un autre. Il pose un cube rouge. Le même geste, deux fois. Tu poses un, puis un ? Oui, papa. La petite tour tient. Merci, Nino. Papa a vu le geste entier. Le ventre de Nino se desserre. Les épaules se relèvent un peu. Elle tient, maman. Tu la vois, ta tour ? Oui, maman. Le cube jaune reste sous le canapé. Je le vois, là. Il attend, sous le bois ? Oui. Nino ne tend pas la main. Il reste près de sa tour. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1633,18 +1652,18 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>118</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.28</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1667,30 +1686,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>répéter</t>
+          <t>cube</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>380</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1699,10 +1718,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1711,44 +1730,42 @@
         <v>50</v>
       </c>
       <c r="AU4" s="2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=un_cube_puis_un_autre; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Nino va près du canapé.
-narrateur|Il parle tout doux.
+          <t>narrateur|Nino referme la bouche.
+narrateur|Il refuse de tout prendre.
+narrateur|Personne ne parle.
+narrateur|Il observe un cube bleu.
+narrateur|Il écoute le salon, un instant.
 enfant-m|Un cube.
+narrateur|Nino pose le cube bleu.
+narrateur|Le tapis le tient.
 enfant-m|Puis un autre.
-enfant-m|Tout doux.
-maman|Tu as su répéter.
-narrateur|Victorina écoute.
-narrateur|Elle va observer d'abord.
-narrateur|Nino pose un cube bleu.
-narrateur|Le cube fait un petit bruit.
-narrateur|Victorina regarde.
-maman|Observer d'abord, c'est possible.
-narrateur|Nino pose un cube vert.
-narrateur|La tour monte un peu.
-narrateur|Plus tard, Victorina tend la main.
-narrateur|Elle pose le cube rouge.
-enfant-m|Encore un.
-narrateur|Nino glisse le cube jaune.
-narrateur|Celui du canapé.
-narrateur|Il le pose tout en haut.
-narrateur|La tour touche le rayon.
-maman|Bravo, Nino.
-maman|Tu as laissé le temps.
-enfant-m|Elle touche la lumière.
-maman|Oui.
-narrateur|Le cube jaune brille un peu.
-narrateur|Victorina pose une main à plat.
-enfant-m|On n'avance plus.
-maman|On regarde, maintenant.</t>
+narrateur|Il pose un cube rouge.
+narrateur|Le même geste, deux fois.
+papa|Tu poses un, puis un ?
+enfant-m|Oui, papa.
+narrateur|La petite tour tient.
+papa|Merci, Nino.
+narrateur|Papa a vu le geste entier.
+narrateur|Le ventre de Nino se desserre.
+narrateur|Les épaules se relèvent un peu.
+enfant-m|Elle tient, maman.
+maman|Tu la vois, ta tour ?
+enfant-m|Oui, maman.
+narrateur|Le cube jaune reste sous le canapé.
+enfant-m|Je le vois, là.
+maman|Il attend, sous le bois ?
+enfant-m|Oui.
+narrateur|Nino ne tend pas la main.
+narrateur|Il reste près de sa tour.</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr">
@@ -1780,17 +1797,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Le doudou a encore l'oreille dehors. Je rentre. C'est une belle tour. Elle touche le rayon. Le cube jaune est le toit. Victorina a regardé d'abord. Nino a répété. Tu as fini de ranger tes cubes ? Oui, maman. Victorina range le cube rouge. Nino range le bleu. Le jaune aussi. Le tapis redevient plat. L'horloge fait tic-tac, encore. Le cacao n'est plus dans l'air. Le doudou attend toujours. Je le mets sur le canapé. Voilà. L'oreille n'est plus coincée. Il est avec nous. Oui. Sur le coussin.</t>
+          <t>Je le veux, maintenant ! Nino se penche sous le canapé. Sa main part trop vite. Le cube jaune glisse plus loin. Le tapis se plisse, sous les genoux. Oh. Nino s'arrête. Ses mains se ferment, puis s'ouvrent. Nino refuse de foncer. Personne ne parle. Il observe le cube, un instant. Il écoute l'horloge, près du bois. Sous le canapé, l'éclat de cube brille. Il brille, comme tout à l'heure. Tu le vois, toi ? Oui, sur le cube. Nino avance la main, lente. Il regarde le cube. Puis il le prend. Je le tiens. Tu le poses sur la tour ? Oui, maman. Nino pose le cube jaune. Le même geste, une fois de plus. La tour tient, plus haute.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Le doudou a encore l'oreille dehors. Je rentre. C'est une belle tour. Elle touche le rayon. Le cube jaune est le toit. Victorina a regardé d'abord. Nino a répété. Tu as fini de ranger tes cubes ? Oui, maman. Victorina range le cube rouge. Nino range le bleu. Le jaune aussi. Le tapis redevient plat. L'horloge fait tic-tac, encore. Le cacao n'est plus dans l'air. Le doudou attend toujours. Je le mets sur le canapé. Voilà. L'oreille n'est plus coincée. Il est avec nous. Oui. Sur le coussin.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Je le veux, maintenant ! Nino se penche sous le canapé. Sa main part trop vite. Le cube jaune glisse plus loin. Le tapis se plisse, sous les genoux. Oh. Nino s'arrête. Ses mains se ferment, puis s'ouvrent. Nino refuse de foncer. Personne ne parle. Il observe le cube, un instant. Il écoute l'horloge, près du bois. Sous le canapé, l'&lt;emphasis level="moderate"&gt;éclat de cube&lt;/emphasis&gt; brille. Il brille, comme tout à l'heure. Tu le vois, toi ? Oui, sur le cube. Nino avance la main, lente. Il regarde le cube. Puis il le prend. Je le tiens. Tu le poses sur la tour ? Oui, maman. Nino pose le cube jaune. Le même geste, une fois de plus. La tour tient, plus haute.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Bérénice range un cube. Maman sourit.&lt;/slow&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Je le veux, maintenant ! Nino se penche sous le canapé. Sa main part trop vite. Le cube jaune glisse plus loin. Le tapis se plisse, sous les genoux. Oh. Nino s'arrête. Ses mains se ferment, puis s'ouvrent. Nino refuse de foncer. Personne ne parle. Il observe le cube, un instant. Il écoute l'horloge, près du bois. Sous le canapé, l'&lt;emphasis&gt;éclat de cube&lt;/emphasis&gt; brille. Il brille, comme tout à l'heure. Tu le vois, toi ? Oui, sur le cube. Nino avance la main, lente. Il regarde le cube. Puis il le prend. Je le tiens. Tu le poses sur la tour ? Oui, maman. Nino pose le cube jaune. Le même geste, une fois de plus. La tour tient, plus haute.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1837,30 +1854,34 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>118</v>
+        <v>134</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.93</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.28</v>
+        <v>1.18</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AE5" s="2" t="inlineStr"/>
+          <t>-2st</t>
+        </is>
+      </c>
+      <c r="AE5" s="2" t="inlineStr">
+        <is>
+          <t>low-pitch</t>
+        </is>
+      </c>
       <c r="AF5" s="2" t="inlineStr">
         <is>
           <t>medium</t>
@@ -1869,28 +1890,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat de cube</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>520</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>380</v>
+        <v>300</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>tense</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1899,50 +1924,57 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.93</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.93</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
       </c>
       <c r="AT5" s="2" t="n">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="AU5" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=obstacle; intention=alerter_sans_effrayer; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=il_refuse_de_foncer_retrouve_l_eclat; tempo=resserré; sourire=aucun; respiration=retenue</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Le doudou a encore l'oreille dehors.
-papa|Je rentre.
-papa|C'est une belle tour.
-enfant-m|Elle touche le rayon.
-papa|Le cube jaune est le toit.
-maman|Victorina a regardé d'abord.
-papa|Nino a répété.
-maman|Tu as fini de ranger tes cubes ?
+          <t>enfant-m|Je le veux, maintenant !
+narrateur|Nino se penche sous le canapé.
+narrateur|Sa main part trop vite.
+narrateur|Le cube jaune glisse plus loin.
+narrateur|Le tapis se plisse, sous les genoux.
+enfant-m|Oh.
+narrateur|Nino s'arrête.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Nino refuse de foncer.
+narrateur|Personne ne parle.
+narrateur|Il observe le cube, un instant.
+narrateur|Il écoute l'horloge, près du bois.
+narrateur|Sous le canapé, l'éclat de cube brille.
+enfant-m|Il brille, comme tout à l'heure.
+papa|Tu le vois, toi ?
+enfant-m|Oui, sur le cube.
+narrateur|Nino avance la main, lente.
+narrateur|Il regarde le cube.
+narrateur|Puis il le prend.
+enfant-m|Je le tiens.
+maman|Tu le poses sur la tour ?
 enfant-m|Oui, maman.
-narrateur|Victorina range le cube rouge.
-narrateur|Nino range le bleu.
-enfant-m|Le jaune aussi.
-papa|Le tapis redevient plat.
-narrateur|L'horloge fait tic-tac, encore.
-narrateur|Le cacao n'est plus dans l'air.
-maman|Le doudou attend toujours.
-enfant-m|Je le mets sur le canapé.
-papa|Voilà.
-narrateur|L'oreille n'est plus coincée.
-enfant-m|Il est avec nous.
-maman|Oui.
-maman|Sur le coussin.</t>
+narrateur|Nino pose le cube jaune.
+narrateur|Le même geste, une fois de plus.
+narrateur|La tour tient, plus haute.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
         <is>
-          <t>cubes,porte</t>
+          <t>cubes</t>
         </is>
       </c>
     </row>
@@ -1969,17 +2001,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le doudou est sur le canapé. La tour n'est plus là. Bonne fin d'après-midi, Nino. Le rayon a bougé.</t>
+          <t>Ils restent assis sur le tapis. Le vent se tait, près du rideau. Tu veux un bout de pain ? Oui, maman. Nino croque. C'est croustillant, un peu chaud. Comme tout à l'heure, papa ! Tu le vois, toi ? Oui, sur le cube. On est bien, ici. Nino pose le pain près de la tour. On le voit, maman. Tu le vois sur le cube ? Oui, l'éclat. La tour se tient sur le tapis. L'horloge pose un tic. Le cube jaune brille, tout en haut. L'éclat de cube tient sur l'arête.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le doudou est sur le canapé. La tour n'est plus là. Bonne fin d'après-midi, Nino. Le rayon a bougé.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent assis sur le tapis. Le vent se tait, près du rideau. Tu veux un bout de pain ? Oui, maman. Nino croque. C'est croustillant, un peu chaud. Comme tout à l'heure, papa ! Tu le vois, toi ? Oui, sur le cube. On est bien, ici. Nino pose le pain près de la tour. On le voit, maman. Tu le vois sur le cube ? Oui, l'éclat. La tour se tient sur le tapis. L'horloge pose un tic. Le cube jaune brille, tout en haut. L'&lt;emphasis level="moderate"&gt;éclat de cube&lt;/emphasis&gt; tient sur l'arête.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent assis sur le tapis. Le vent se tait, près du rideau. Tu veux un bout de pain ? Oui, maman. Nino croque. C'est croustillant, un peu chaud. Comme tout à l'heure, papa ! Tu le vois, toi ? Oui, sur le cube. On est bien, ici. Nino pose le pain près de la tour. On le voit, maman. Tu le vois sur le cube ? Oui, l'éclat. La tour se tient sur le tapis. L'horloge pose un tic. Le cube jaune brille, tout en haut. L'&lt;emphasis&gt;éclat de cube&lt;/emphasis&gt; tient sur l'arête.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2026,7 +2058,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2034,10 +2066,10 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.36</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2046,12 +2078,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2060,17 +2092,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de cube</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>380</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2079,11 +2115,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2092,27 +2128,45 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_l_arete; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|Le doudou est sur le canapé.
-narrateur|La tour n'est plus là.
-maman|Bonne fin d'après-midi, Nino.
-papa|Le rayon a bougé.</t>
+          <t>narrateur|Ils restent assis sur le tapis.
+narrateur|Le vent se tait, près du rideau.
+maman|Tu veux un bout de pain ?
+enfant-m|Oui, maman.
+narrateur|Nino croque.
+narrateur|C'est croustillant, un peu chaud.
+enfant-m|Comme tout à l'heure, papa !
+papa|Tu le vois, toi ?
+enfant-m|Oui, sur le cube.
+maman|On est bien, ici.
+narrateur|Nino pose le pain près de la tour.
+enfant-m|On le voit, maman.
+maman|Tu le vois sur le cube ?
+enfant-m|Oui, l'éclat.
+narrateur|La tour se tient sur le tapis.
+narrateur|L'horloge pose un tic.
+narrateur|Le cube jaune brille, tout en haut.
+narrateur|L'éclat de cube tient sur l'arête.</t>
         </is>
       </c>
     </row>
@@ -2133,7 +2187,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2218,6 +2272,13 @@
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>

<commit_message>
feat(F-NAR-019): ATOM-DIF.BES.001-04 Les cubes de Nino (polish)
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.BES.001-04.xlsx
+++ b/stories/arbres/ATOM-DIF.BES.001-04.xlsx
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Un rayon jaune pose un carré sur le tapis. Le pied du canapé le coupe. Un cube jaune y reste coincé. Sur l'arête, un éclat de cube luit. Il brille, papa. Tu le vois, sur le cube ? Ça sent le pain du goûter. Papa coupe le pain, près de la table. L'horloge fait tic-tac. Le rideau bouge un peu. Un doudou attend sur le canapé. Tu as vu le cube, Nino ? Il est sous le canapé. On le laisse un moment. D'autres cubes sont sur le tapis. Ils sont lisses, un peu froids. Un bleu attend près du pied. Je veux une tour, maintenant ! Aussi haute que le canapé ! Tu la veux vite ? Oui, tout de suite ! En ce moment, Nino prend trop de cubes. Les cubes glissent entre ses doigts. Ça fait clac, sur le tapis. La tour tombe, trop vite. Le cube jaune roule sous le canapé. Oh. L'éclat de cube tremble, puis tient. Le sourire de Nino disparaît. Dans sa poitrine, ça se bouscule. L'envie et l'inquiétude se heurtent. Ça ne veut pas, papa. Ses épaules tombent un peu. Papa se baisse à sa hauteur. Tu regardes les cubes ? Je les veux tous. Tu les prends trop vite, Nino ? Oui, maman. Nino serre les mains, trop fort. Ses doigts restent fermés. Son souffle est court. On regarde un cube ? Un seul ?</t>
+          <t>Un rayon jaune pose un carré sur le tapis. Le pied du canapé coupe le carré jaune. Un cube jaune reste coincé dans le carré. Sur l'arête, un éclat de cube luit. Il brille, papa. Tu le vois, sur le cube ? Ça sent le pain du goûter, chaud. Papa coupe le pain, près de la table. L'horloge fait tic-tac, près du mur. Le rideau bouge un peu, près de la vitre. Un doudou gris attend sur le canapé. Tu as vu le cube, Nino ? Il est près du pied. On le laisse un moment. D'autres cubes sont sur le tapis. Les cubes sont lisses, un peu froids. Un cube bleu attend près du pied. Je veux une tour, maintenant ! Aussi haute que le canapé ! Tu la veux vite ? Oui, tout de suite ! En ce moment, Nino prend trop de cubes. Les cubes glissent entre ses petits doigts. Ça fait clac, fort, sur le tapis. La tour tombe trop vite, sur le tapis. Le cube jaune roule sous le canapé. Oh. L'éclat de cube tremble, puis tient. Le sourire de Nino disparaît d'un coup. Dans sa poitrine, ça se bouscule. L'envie et l'inquiétude se heurtent. Ça ne veut pas, papa. Ses épaules tombent un peu, lourdes. Papa se baisse à la hauteur de Nino. Tu regardes les cubes ? Je les veux tous. Tu les prends trop vite, Nino ? Oui, maman. Nino serre les mains trop fort, contre lui. Ses doigts restent fermés, un peu chauds. Son souffle est court, dans le salon. On regarde un cube ? Un seul ?</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Un rayon jaune pose un carré sur le tapis. Le pied du canapé le coupe. Un cube jaune y reste coincé. Sur l'arête, un &lt;emphasis level="moderate"&gt;éclat de cube&lt;/emphasis&gt; luit. Il brille, papa. Tu le vois, sur le cube ? Ça sent le pain du goûter. Papa coupe le pain, près de la table. L'horloge fait tic-tac. Le rideau bouge un peu. Un doudou attend sur le canapé. Tu as vu le cube, Nino ? Il est sous le canapé. On le laisse un moment. D'autres cubes sont sur le tapis. Ils sont lisses, un peu froids. Un bleu attend près du pied. Je veux une tour, maintenant ! Aussi haute que le canapé ! Tu la veux vite ? Oui, tout de suite ! En ce moment, Nino prend trop de cubes. Les cubes glissent entre ses doigts. Ça fait clac, sur le tapis. La tour tombe, trop vite. Le cube jaune roule sous le canapé. Oh. L'éclat de cube tremble, puis tient. Le sourire de Nino disparaît. Dans sa poitrine, ça se bouscule. L'envie et l'inquiétude se heurtent. Ça ne veut pas, papa. Ses épaules tombent un peu. Papa se baisse à sa hauteur. Tu regardes les cubes ? Je les veux tous. Tu les prends trop vite, Nino ? Oui, maman. Nino serre les mains, trop fort. Ses doigts restent fermés. Son souffle est court. On regarde un cube ? Un seul ?&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Un rayon jaune pose un carré sur le tapis. Le pied du canapé coupe le carré jaune. Un cube jaune reste coincé dans le carré. Sur l'arête, un &lt;emphasis level="moderate"&gt;éclat de cube&lt;/emphasis&gt; luit. Il brille, papa. Tu le vois, sur le cube ? Ça sent le pain du goûter, chaud. Papa coupe le pain, près de la table. L'horloge fait tic-tac, près du mur. Le rideau bouge un peu, près de la vitre. Un doudou gris attend sur le canapé. Tu as vu le cube, Nino ? Il est près du pied. On le laisse un moment. D'autres cubes sont sur le tapis. Les cubes sont lisses, un peu froids. Un cube bleu attend près du pied. Je veux une tour, maintenant ! Aussi haute que le canapé ! Tu la veux vite ? Oui, tout de suite ! En ce moment, Nino prend trop de cubes. Les cubes glissent entre ses petits doigts. Ça fait clac, fort, sur le tapis. La tour tombe trop vite, sur le tapis. Le cube jaune roule sous le canapé. Oh. L'éclat de cube tremble, puis tient. Le sourire de Nino disparaît d'un coup. Dans sa poitrine, ça se bouscule. L'envie et l'inquiétude se heurtent. Ça ne veut pas, papa. Ses épaules tombent un peu, lourdes. Papa se baisse à la hauteur de Nino. Tu regardes les cubes ? Je les veux tous. Tu les prends trop vite, Nino ? Oui, maman. Nino serre les mains trop fort, contre lui. Ses doigts restent fermés, un peu chauds. Son souffle est court, dans le salon. On regarde un cube ? Un seul ?&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Un rayon jaune pose un carré sur le tapis. Le pied du canapé le coupe. Un cube jaune y reste coincé. Sur l'arête, un &lt;emphasis&gt;éclat de cube&lt;/emphasis&gt; luit. Il brille, papa. Tu le vois, sur le cube ? Ça sent le pain du goûter. Papa coupe le pain, près de la table. L'horloge fait tic-tac. Le rideau bouge un peu. Un doudou attend sur le canapé. Tu as vu le cube, Nino ? Il est sous le canapé. On le laisse un moment. D'autres cubes sont sur le tapis. Ils sont lisses, un peu froids. Un bleu attend près du pied. Je veux une tour, maintenant ! Aussi haute que le canapé ! Tu la veux vite ? Oui, tout de suite ! En ce moment, Nino prend trop de cubes. Les cubes glissent entre ses doigts. Ça fait clac, sur le tapis. La tour tombe, trop vite. Le cube jaune roule sous le canapé. Oh. L'éclat de cube tremble, puis tient. Le sourire de Nino disparaît. Dans sa poitrine, ça se bouscule. L'envie et l'inquiétude se heurtent. Ça ne veut pas, papa. Ses épaules tombent un peu. Papa se baisse à sa hauteur. Tu regardes les cubes ? Je les veux tous. Tu les prends trop vite, Nino ? Oui, maman. Nino serre les mains, trop fort. Ses doigts restent fermés. Son souffle est court. On regarde un cube ? Un seul ? [pause]</t>
+          <t>Un rayon jaune pose un carré sur le tapis. Le pied du canapé coupe le carré jaune. Un cube jaune reste coincé dans le carré. Sur l'arête, un &lt;emphasis&gt;éclat de cube&lt;/emphasis&gt; luit. Il brille, papa. Tu le vois, sur le cube ? Ça sent le pain du goûter, chaud. Papa coupe le pain, près de la table. L'horloge fait tic-tac, près du mur. Le rideau bouge un peu, près de la vitre. Un doudou gris attend sur le canapé. Tu as vu le cube, Nino ? Il est près du pied. On le laisse un moment. D'autres cubes sont sur le tapis. Les cubes sont lisses, un peu froids. Un cube bleu attend près du pied. Je veux une tour, maintenant ! Aussi haute que le canapé ! Tu la veux vite ? Oui, tout de suite ! En ce moment, Nino prend trop de cubes. Les cubes glissent entre ses petits doigts. Ça fait clac, fort, sur le tapis. La tour tombe trop vite, sur le tapis. Le cube jaune roule sous le canapé. Oh. L'éclat de cube tremble, puis tient. Le sourire de Nino disparaît d'un coup. Dans sa poitrine, ça se bouscule. L'envie et l'inquiétude se heurtent. Ça ne veut pas, papa. Ses épaules tombent un peu, lourdes. Papa se baisse à la hauteur de Nino. Tu regardes les cubes ? Je les veux tous. Tu les prends trop vite, Nino ? Oui, maman. Nino serre les mains trop fort, contre lui. Ses doigts restent fermés, un peu chauds. Son souffle est court, dans le salon. On regarde un cube ? Un seul ? [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1334,46 +1334,46 @@
       <c r="AW2" t="inlineStr">
         <is>
           <t>narrateur|Un rayon jaune pose un carré sur le tapis.
-narrateur|Le pied du canapé le coupe.
-narrateur|Un cube jaune y reste coincé.
+narrateur|Le pied du canapé coupe le carré jaune.
+narrateur|Un cube jaune reste coincé dans le carré.
 narrateur|Sur l'arête, un éclat de cube luit.
 enfant-m|Il brille, papa.
 papa|Tu le vois, sur le cube ?
-narrateur|Ça sent le pain du goûter.
+narrateur|Ça sent le pain du goûter, chaud.
 narrateur|Papa coupe le pain, près de la table.
-narrateur|L'horloge fait tic-tac.
-narrateur|Le rideau bouge un peu.
-narrateur|Un doudou attend sur le canapé.
+narrateur|L'horloge fait tic-tac, près du mur.
+narrateur|Le rideau bouge un peu, près de la vitre.
+narrateur|Un doudou gris attend sur le canapé.
 maman|Tu as vu le cube, Nino ?
-enfant-m|Il est sous le canapé.
+enfant-m|Il est près du pied.
 maman|On le laisse un moment.
 narrateur|D'autres cubes sont sur le tapis.
-narrateur|Ils sont lisses, un peu froids.
-narrateur|Un bleu attend près du pied.
+narrateur|Les cubes sont lisses, un peu froids.
+narrateur|Un cube bleu attend près du pied.
 enfant-m|Je veux une tour, maintenant !
 enfant-m|Aussi haute que le canapé !
 papa|Tu la veux vite ?
 enfant-m|Oui, tout de suite !
 narrateur|En ce moment, Nino prend trop de cubes.
-narrateur|Les cubes glissent entre ses doigts.
-narrateur|Ça fait clac, sur le tapis.
-narrateur|La tour tombe, trop vite.
+narrateur|Les cubes glissent entre ses petits doigts.
+narrateur|Ça fait clac, fort, sur le tapis.
+narrateur|La tour tombe trop vite, sur le tapis.
 narrateur|Le cube jaune roule sous le canapé.
 enfant-m|Oh.
 narrateur|L'éclat de cube tremble, puis tient.
-narrateur|Le sourire de Nino disparaît.
+narrateur|Le sourire de Nino disparaît d'un coup.
 narrateur|Dans sa poitrine, ça se bouscule.
 narrateur|L'envie et l'inquiétude se heurtent.
 enfant-m|Ça ne veut pas, papa.
-narrateur|Ses épaules tombent un peu.
-narrateur|Papa se baisse à sa hauteur.
+narrateur|Ses épaules tombent un peu, lourdes.
+narrateur|Papa se baisse à la hauteur de Nino.
 papa|Tu regardes les cubes ?
 enfant-m|Je les veux tous.
 maman|Tu les prends trop vite, Nino ?
 enfant-m|Oui, maman.
-narrateur|Nino serre les mains, trop fort.
-narrateur|Ses doigts restent fermés.
-narrateur|Son souffle est court.
+narrateur|Nino serre les mains trop fort, contre lui.
+narrateur|Ses doigts restent fermés, un peu chauds.
+narrateur|Son souffle est court, dans le salon.
 papa|On regarde un cube ?
 enfant-m|Un seul ?</t>
         </is>
@@ -1595,17 +1595,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Nino referme la bouche. Il refuse de tout prendre. Personne ne parle. Il observe un cube bleu. Il écoute le salon, un instant. Un cube. Nino pose le cube bleu. Le tapis le tient. Puis un autre. Il pose un cube rouge. Le même geste, deux fois. Tu poses un, puis un ? Oui, papa. La petite tour tient. Merci, Nino. Papa a vu le geste entier. Le ventre de Nino se desserre. Les épaules se relèvent un peu. Elle tient, maman. Tu la vois, ta tour ? Oui, maman. Le cube jaune reste sous le canapé. Je le vois, là. Il attend, sous le bois ? Oui. Nino ne tend pas la main. Il reste près de sa tour.</t>
+          <t>Nino referme la bouche, un moment. Il refuse de tout prendre d'un coup. Personne ne parle, dans le salon. Il observe un cube bleu, posé là. Il écoute le salon, un instant. Un cube. Nino pose le cube bleu sur le tapis. Le tapis tient le cube, sans bouger. Puis un autre. Il pose un cube rouge, au-dessus. Il refait le même geste, deux fois. Tu poses un, puis un ? Oui, papa. La petite tour tient, bien droite. Merci, Nino. Papa a vu le geste entier, sans parler. Le ventre de Nino se desserre un peu. Les épaules de Nino se relèvent un peu. Elle tient, maman. Tu la vois, ta tour ? Oui, maman. Le cube jaune reste sous le canapé. Je le vois, là. Il attend, sous le bois ? Oui. Nino ne tend pas la main, cette fois. Il reste près de sa petite tour.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino referme la bouche. Il refuse de tout prendre. Personne ne parle. Il observe un &lt;emphasis level="moderate"&gt;cube&lt;/emphasis&gt; bleu. Il écoute le salon, un instant. Un cube. Nino pose le cube bleu. Le tapis le tient. Puis un autre. Il pose un cube rouge. Le même geste, deux fois. Tu poses un, puis un ? Oui, papa. La petite tour tient. Merci, Nino. Papa a vu le geste entier. Le ventre de Nino se desserre. Les épaules se relèvent un peu. Elle tient, maman. Tu la vois, ta tour ? Oui, maman. Le cube jaune reste sous le canapé. Je le vois, là. Il attend, sous le bois ? Oui. Nino ne tend pas la main. Il reste près de sa tour.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino referme la bouche, un moment. Il refuse de tout prendre d'un coup. Personne ne parle, dans le salon. Il observe un &lt;emphasis level="moderate"&gt;cube&lt;/emphasis&gt; bleu, posé là. Il écoute le salon, un instant. Un cube. Nino pose le cube bleu sur le tapis. Le tapis tient le cube, sans bouger. Puis un autre. Il pose un cube rouge, au-dessus. Il refait le même geste, deux fois. Tu poses un, puis un ? Oui, papa. La petite tour tient, bien droite. Merci, Nino. Papa a vu le geste entier, sans parler. Le ventre de Nino se desserre un peu. Les épaules de Nino se relèvent un peu. Elle tient, maman. Tu la vois, ta tour ? Oui, maman. Le cube jaune reste sous le canapé. Je le vois, là. Il attend, sous le bois ? Oui. Nino ne tend pas la main, cette fois. Il reste près de sa petite tour.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Nino referme la bouche. Il refuse de tout prendre. Personne ne parle. Il observe un &lt;emphasis&gt;cube&lt;/emphasis&gt; bleu. Il écoute le salon, un instant. Un cube. Nino pose le cube bleu. Le tapis le tient. Puis un autre. Il pose un cube rouge. Le même geste, deux fois. Tu poses un, puis un ? Oui, papa. La petite tour tient. Merci, Nino. Papa a vu le geste entier. Le ventre de Nino se desserre. Les épaules se relèvent un peu. Elle tient, maman. Tu la vois, ta tour ? Oui, maman. Le cube jaune reste sous le canapé. Je le vois, là. Il attend, sous le bois ? Oui. Nino ne tend pas la main. Il reste près de sa tour. [pause]</t>
+          <t>Nino referme la bouche, un moment. Il refuse de tout prendre d'un coup. Personne ne parle, dans le salon. Il observe un &lt;emphasis&gt;cube&lt;/emphasis&gt; bleu, posé là. Il écoute le salon, un instant. Un cube. Nino pose le cube bleu sur le tapis. Le tapis tient le cube, sans bouger. Puis un autre. Il pose un cube rouge, au-dessus. Il refait le même geste, deux fois. Tu poses un, puis un ? Oui, papa. La petite tour tient, bien droite. Merci, Nino. Papa a vu le geste entier, sans parler. Le ventre de Nino se desserre un peu. Les épaules de Nino se relèvent un peu. Elle tient, maman. Tu la vois, ta tour ? Oui, maman. Le cube jaune reste sous le canapé. Je le vois, là. Il attend, sous le bois ? Oui. Nino ne tend pas la main, cette fois. Il reste près de sa petite tour. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1739,24 +1739,24 @@
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Nino referme la bouche.
-narrateur|Il refuse de tout prendre.
-narrateur|Personne ne parle.
-narrateur|Il observe un cube bleu.
+          <t>narrateur|Nino referme la bouche, un moment.
+narrateur|Il refuse de tout prendre d'un coup.
+narrateur|Personne ne parle, dans le salon.
+narrateur|Il observe un cube bleu, posé là.
 narrateur|Il écoute le salon, un instant.
 enfant-m|Un cube.
-narrateur|Nino pose le cube bleu.
-narrateur|Le tapis le tient.
+narrateur|Nino pose le cube bleu sur le tapis.
+narrateur|Le tapis tient le cube, sans bouger.
 enfant-m|Puis un autre.
-narrateur|Il pose un cube rouge.
-narrateur|Le même geste, deux fois.
+narrateur|Il pose un cube rouge, au-dessus.
+narrateur|Il refait le même geste, deux fois.
 papa|Tu poses un, puis un ?
 enfant-m|Oui, papa.
-narrateur|La petite tour tient.
+narrateur|La petite tour tient, bien droite.
 papa|Merci, Nino.
-narrateur|Papa a vu le geste entier.
-narrateur|Le ventre de Nino se desserre.
-narrateur|Les épaules se relèvent un peu.
+narrateur|Papa a vu le geste entier, sans parler.
+narrateur|Le ventre de Nino se desserre un peu.
+narrateur|Les épaules de Nino se relèvent un peu.
 enfant-m|Elle tient, maman.
 maman|Tu la vois, ta tour ?
 enfant-m|Oui, maman.
@@ -1764,8 +1764,8 @@
 enfant-m|Je le vois, là.
 maman|Il attend, sous le bois ?
 enfant-m|Oui.
-narrateur|Nino ne tend pas la main.
-narrateur|Il reste près de sa tour.</t>
+narrateur|Nino ne tend pas la main, cette fois.
+narrateur|Il reste près de sa petite tour.</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr">
@@ -1797,17 +1797,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Je le veux, maintenant ! Nino se penche sous le canapé. Sa main part trop vite. Le cube jaune glisse plus loin. Le tapis se plisse, sous les genoux. Oh. Nino s'arrête. Ses mains se ferment, puis s'ouvrent. Nino refuse de foncer. Personne ne parle. Il observe le cube, un instant. Il écoute l'horloge, près du bois. Sous le canapé, l'éclat de cube brille. Il brille, comme tout à l'heure. Tu le vois, toi ? Oui, sur le cube. Nino avance la main, lente. Il regarde le cube. Puis il le prend. Je le tiens. Tu le poses sur la tour ? Oui, maman. Nino pose le cube jaune. Le même geste, une fois de plus. La tour tient, plus haute.</t>
+          <t>Je le veux, maintenant ! Nino se penche sous le canapé, vite. Sa main part trop vite, sous le bois. Le cube jaune glisse plus loin, sous l'ombre. Le tapis se plisse, sous les genoux. Oh. Nino s'arrête, les genoux au tapis. Ses mains se ferment, puis s'ouvrent. Nino refuse de foncer, cette fois. Personne ne dit la suite, sous le bois. Il observe le cube jaune, un instant. Il écoute l'horloge, près du bois. Sous le canapé, l'éclat de cube brille. Il brille, comme tout à l'heure. Tu le vois, toi ? Oui, sur le cube. Nino avance la main, lente, ouverte. Il regarde le cube, sans presser. Puis il le prend, sans tirer. Je le tiens. Tu le poses sur la tour ? Oui, maman. Nino pose le cube jaune, tout en haut. Le même geste, une fois de plus. La tour tient, plus haute, sur le tapis.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Je le veux, maintenant ! Nino se penche sous le canapé. Sa main part trop vite. Le cube jaune glisse plus loin. Le tapis se plisse, sous les genoux. Oh. Nino s'arrête. Ses mains se ferment, puis s'ouvrent. Nino refuse de foncer. Personne ne parle. Il observe le cube, un instant. Il écoute l'horloge, près du bois. Sous le canapé, l'&lt;emphasis level="moderate"&gt;éclat de cube&lt;/emphasis&gt; brille. Il brille, comme tout à l'heure. Tu le vois, toi ? Oui, sur le cube. Nino avance la main, lente. Il regarde le cube. Puis il le prend. Je le tiens. Tu le poses sur la tour ? Oui, maman. Nino pose le cube jaune. Le même geste, une fois de plus. La tour tient, plus haute.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Je le veux, maintenant ! Nino se penche sous le canapé, vite. Sa main part trop vite, sous le bois. Le cube jaune glisse plus loin, sous l'ombre. Le tapis se plisse, sous les genoux. Oh. Nino s'arrête, les genoux au tapis. Ses mains se ferment, puis s'ouvrent. Nino refuse de foncer, cette fois. Personne ne dit la suite, sous le bois. Il observe le cube jaune, un instant. Il écoute l'horloge, près du bois. Sous le canapé, l'&lt;emphasis level="moderate"&gt;éclat de cube&lt;/emphasis&gt; brille. Il brille, comme tout à l'heure. Tu le vois, toi ? Oui, sur le cube. Nino avance la main, lente, ouverte. Il regarde le cube, sans presser. Puis il le prend, sans tirer. Je le tiens. Tu le poses sur la tour ? Oui, maman. Nino pose le cube jaune, tout en haut. Le même geste, une fois de plus. La tour tient, plus haute, sur le tapis.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Je le veux, maintenant ! Nino se penche sous le canapé. Sa main part trop vite. Le cube jaune glisse plus loin. Le tapis se plisse, sous les genoux. Oh. Nino s'arrête. Ses mains se ferment, puis s'ouvrent. Nino refuse de foncer. Personne ne parle. Il observe le cube, un instant. Il écoute l'horloge, près du bois. Sous le canapé, l'&lt;emphasis&gt;éclat de cube&lt;/emphasis&gt; brille. Il brille, comme tout à l'heure. Tu le vois, toi ? Oui, sur le cube. Nino avance la main, lente. Il regarde le cube. Puis il le prend. Je le tiens. Tu le poses sur la tour ? Oui, maman. Nino pose le cube jaune. Le même geste, une fois de plus. La tour tient, plus haute.&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Je le veux, maintenant ! Nino se penche sous le canapé, vite. Sa main part trop vite, sous le bois. Le cube jaune glisse plus loin, sous l'ombre. Le tapis se plisse, sous les genoux. Oh. Nino s'arrête, les genoux au tapis. Ses mains se ferment, puis s'ouvrent. Nino refuse de foncer, cette fois. Personne ne dit la suite, sous le bois. Il observe le cube jaune, un instant. Il écoute l'horloge, près du bois. Sous le canapé, l'&lt;emphasis&gt;éclat de cube&lt;/emphasis&gt; brille. Il brille, comme tout à l'heure. Tu le vois, toi ? Oui, sur le cube. Nino avance la main, lente, ouverte. Il regarde le cube, sans presser. Puis il le prend, sans tirer. Je le tiens. Tu le poses sur la tour ? Oui, maman. Nino pose le cube jaune, tout en haut. Le même geste, une fois de plus. La tour tient, plus haute, sur le tapis.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1946,30 +1946,30 @@
       <c r="AW5" t="inlineStr">
         <is>
           <t>enfant-m|Je le veux, maintenant !
-narrateur|Nino se penche sous le canapé.
-narrateur|Sa main part trop vite.
-narrateur|Le cube jaune glisse plus loin.
+narrateur|Nino se penche sous le canapé, vite.
+narrateur|Sa main part trop vite, sous le bois.
+narrateur|Le cube jaune glisse plus loin, sous l'ombre.
 narrateur|Le tapis se plisse, sous les genoux.
 enfant-m|Oh.
-narrateur|Nino s'arrête.
+narrateur|Nino s'arrête, les genoux au tapis.
 narrateur|Ses mains se ferment, puis s'ouvrent.
-narrateur|Nino refuse de foncer.
-narrateur|Personne ne parle.
-narrateur|Il observe le cube, un instant.
+narrateur|Nino refuse de foncer, cette fois.
+narrateur|Personne ne dit la suite, sous le bois.
+narrateur|Il observe le cube jaune, un instant.
 narrateur|Il écoute l'horloge, près du bois.
 narrateur|Sous le canapé, l'éclat de cube brille.
 enfant-m|Il brille, comme tout à l'heure.
 papa|Tu le vois, toi ?
 enfant-m|Oui, sur le cube.
-narrateur|Nino avance la main, lente.
-narrateur|Il regarde le cube.
-narrateur|Puis il le prend.
+narrateur|Nino avance la main, lente, ouverte.
+narrateur|Il regarde le cube, sans presser.
+narrateur|Puis il le prend, sans tirer.
 enfant-m|Je le tiens.
 maman|Tu le poses sur la tour ?
 enfant-m|Oui, maman.
-narrateur|Nino pose le cube jaune.
+narrateur|Nino pose le cube jaune, tout en haut.
 narrateur|Le même geste, une fois de plus.
-narrateur|La tour tient, plus haute.</t>
+narrateur|La tour tient, plus haute, sur le tapis.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
@@ -2001,17 +2001,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Ils restent assis sur le tapis. Le vent se tait, près du rideau. Tu veux un bout de pain ? Oui, maman. Nino croque. C'est croustillant, un peu chaud. Comme tout à l'heure, papa ! Tu le vois, toi ? Oui, sur le cube. On est bien, ici. Nino pose le pain près de la tour. On le voit, maman. Tu le vois sur le cube ? Oui, l'éclat. La tour se tient sur le tapis. L'horloge pose un tic. Le cube jaune brille, tout en haut. L'éclat de cube tient sur l'arête.</t>
+          <t>Ils restent assis sur le tapis, près de la tour. Le vent se tait, près du rideau. Tu veux un bout de pain ? Oui, maman. Nino croque un bout de pain, tiède. C'est croustillant, un peu chaud sous la langue. Comme tout à l'heure, papa ! Tu le vois, toi ? Oui, sur le cube. On est bien, ici. Nino pose le pain près de la tour. On le voit, maman. Tu le vois sur le cube ? Oui, l'éclat. La tour se tient sur le tapis. L'horloge pose un tic, près du mur. Le cube jaune brille, tout en haut. L'éclat de cube tient sur l'arête.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent assis sur le tapis. Le vent se tait, près du rideau. Tu veux un bout de pain ? Oui, maman. Nino croque. C'est croustillant, un peu chaud. Comme tout à l'heure, papa ! Tu le vois, toi ? Oui, sur le cube. On est bien, ici. Nino pose le pain près de la tour. On le voit, maman. Tu le vois sur le cube ? Oui, l'éclat. La tour se tient sur le tapis. L'horloge pose un tic. Le cube jaune brille, tout en haut. L'&lt;emphasis level="moderate"&gt;éclat de cube&lt;/emphasis&gt; tient sur l'arête.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent assis sur le tapis, près de la tour. Le vent se tait, près du rideau. Tu veux un bout de pain ? Oui, maman. Nino croque un bout de pain, tiède. C'est croustillant, un peu chaud sous la langue. Comme tout à l'heure, papa ! Tu le vois, toi ? Oui, sur le cube. On est bien, ici. Nino pose le pain près de la tour. On le voit, maman. Tu le vois sur le cube ? Oui, l'éclat. La tour se tient sur le tapis. L'horloge pose un tic, près du mur. Le cube jaune brille, tout en haut. L'&lt;emphasis level="moderate"&gt;éclat de cube&lt;/emphasis&gt; tient sur l'arête.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent assis sur le tapis. Le vent se tait, près du rideau. Tu veux un bout de pain ? Oui, maman. Nino croque. C'est croustillant, un peu chaud. Comme tout à l'heure, papa ! Tu le vois, toi ? Oui, sur le cube. On est bien, ici. Nino pose le pain près de la tour. On le voit, maman. Tu le vois sur le cube ? Oui, l'éclat. La tour se tient sur le tapis. L'horloge pose un tic. Le cube jaune brille, tout en haut. L'&lt;emphasis&gt;éclat de cube&lt;/emphasis&gt; tient sur l'arête.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent assis sur le tapis, près de la tour. Le vent se tait, près du rideau. Tu veux un bout de pain ? Oui, maman. Nino croque un bout de pain, tiède. C'est croustillant, un peu chaud sous la langue. Comme tout à l'heure, papa ! Tu le vois, toi ? Oui, sur le cube. On est bien, ici. Nino pose le pain près de la tour. On le voit, maman. Tu le vois sur le cube ? Oui, l'éclat. La tour se tient sur le tapis. L'horloge pose un tic, près du mur. Le cube jaune brille, tout en haut. L'&lt;emphasis&gt;éclat de cube&lt;/emphasis&gt; tient sur l'arête.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2149,12 +2149,12 @@
       </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|Ils restent assis sur le tapis.
+          <t>narrateur|Ils restent assis sur le tapis, près de la tour.
 narrateur|Le vent se tait, près du rideau.
 maman|Tu veux un bout de pain ?
 enfant-m|Oui, maman.
-narrateur|Nino croque.
-narrateur|C'est croustillant, un peu chaud.
+narrateur|Nino croque un bout de pain, tiède.
+narrateur|C'est croustillant, un peu chaud sous la langue.
 enfant-m|Comme tout à l'heure, papa !
 papa|Tu le vois, toi ?
 enfant-m|Oui, sur le cube.
@@ -2164,7 +2164,7 @@
 maman|Tu le vois sur le cube ?
 enfant-m|Oui, l'éclat.
 narrateur|La tour se tient sur le tapis.
-narrateur|L'horloge pose un tic.
+narrateur|L'horloge pose un tic, près du mur.
 narrateur|Le cube jaune brille, tout en haut.
 narrateur|L'éclat de cube tient sur l'arête.</t>
         </is>
@@ -2187,7 +2187,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2279,6 +2279,13 @@
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>